<commit_message>
Added excel sheets and organized microscopy data
</commit_message>
<xml_diff>
--- a/data/normalized/basidiospore.xlsx
+++ b/data/normalized/basidiospore.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hensley/Desktop/wiscam_microscopy/data/normalized/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{267F596A-9EEB-CB40-8A2C-FE4D3EEEB04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3D2CC4-57AA-604C-9A84-E6AFDD544CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-33300" yWindow="-1320" windowWidth="27640" windowHeight="16640" xr2:uid="{8188D9C6-D56A-8E47-B77A-6198909A1C26}"/>
   </bookViews>
@@ -812,45 +812,6 @@
       <c r="C2" t="s">
         <v>14</v>
       </c>
-      <c r="D2">
-        <v>25</v>
-      </c>
-      <c r="E2">
-        <v>7.5</v>
-      </c>
-      <c r="F2">
-        <v>8</v>
-      </c>
-      <c r="G2">
-        <v>12</v>
-      </c>
-      <c r="H2">
-        <v>14.5</v>
-      </c>
-      <c r="I2">
-        <v>7</v>
-      </c>
-      <c r="J2">
-        <v>8</v>
-      </c>
-      <c r="K2">
-        <v>12</v>
-      </c>
-      <c r="L2">
-        <v>12</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2">
-        <v>1.5</v>
-      </c>
-      <c r="P2">
-        <v>1</v>
-      </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3">
@@ -861,45 +822,6 @@
       </c>
       <c r="C3" t="s">
         <v>14</v>
-      </c>
-      <c r="D3">
-        <v>25</v>
-      </c>
-      <c r="E3">
-        <v>8</v>
-      </c>
-      <c r="F3">
-        <v>9</v>
-      </c>
-      <c r="G3">
-        <v>11.5</v>
-      </c>
-      <c r="H3">
-        <v>12</v>
-      </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3">
-        <v>7</v>
-      </c>
-      <c r="K3">
-        <v>10</v>
-      </c>
-      <c r="L3">
-        <v>10</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>1.2</v>
-      </c>
-      <c r="O3">
-        <v>1.5</v>
-      </c>
-      <c r="P3">
-        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">

</xml_diff>